<commit_message>
Sync Meetings/Calendar, sidebar rebrand, and all pending work
</commit_message>
<xml_diff>
--- a/JAIN-E Signups, Accountability & Legal Report.xlsx
+++ b/JAIN-E Signups, Accountability & Legal Report.xlsx
@@ -11,10 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accountability" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legal" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Signups'!$A$4:$F$66</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Accountability'!$A$4:$F$66</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -31,34 +28,27 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="000A2640"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <i val="1"/>
       <color rgb="00475569"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
       <sz val="10.5"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <sz val="10.5"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00B91C1C"/>
       <sz val="11"/>
@@ -78,11 +68,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
@@ -91,8 +76,13 @@
         <fgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -100,57 +90,26 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -537,7 +496,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-20 10:34 UTC · 62 accounts with a login (auth) · rows with blank Department/Level/Tabs have signed up but have not yet been provisioned in Control Panel</t>
+          <t>Generated 2026-07-22 06:33 UTC · 62 accounts with a login (auth) · rows with blank Department/Level/Tabs have signed up but have not yet been provisioned in Control Panel</t>
         </is>
       </c>
     </row>
@@ -606,32 +565,32 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Rishi Jain</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>rishi@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Management</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, gtd, crm, projects, construction, inventory, procurement, maintenance, inspection, hr, recruitment, finance, legal, compliance, campaigns, scaling, playbook, documents, video, helpdesk, reports, customer, supplier, whatsapp, mail, settings</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>2026-06-29 06:18 UTC</t>
         </is>
@@ -670,32 +629,32 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>v c</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>vc@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Management</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, gtd, crm, projects, construction, inventory, procurement, maintenance, inspection, hr, recruitment, finance, legal, compliance, campaigns, scaling, playbook, documents, video, helpdesk, reports, customer, supplier, whatsapp, mail, settings</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>2026-06-29 08:28 UTC</t>
         </is>
@@ -734,32 +693,32 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Akashnil Basu</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>socialmedia@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, crm, projects, hr, campaigns, scaling, documents, video, helpdesk, reports, customer, settings</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>2026-06-30 06:01 UTC</t>
         </is>
@@ -798,32 +757,32 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Santanu Naskar</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>projectmanager1@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, inspection, settings</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>2026-07-02 07:19 UTC</t>
         </is>
@@ -862,32 +821,32 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Santanu Goswami</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>dgm.project@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, construction, inventory, procurement, maintenance, inspection, recruitment, documents, video, helpdesk, reports, supplier, settings</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>2026-07-03 09:44 UTC</t>
         </is>
@@ -926,32 +885,32 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Uzma Ahmed</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>career@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, crm, projects, inspection, hr, recruitment, documents, video, helpdesk, reports, settings</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>2026-07-03 11:20 UTC</t>
         </is>
@@ -990,32 +949,32 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Amirul SK</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>graphicsdesinger3.thejaingroup@gmail.com</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, recruitment, campaigns, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>2026-07-07 05:43 UTC</t>
         </is>
@@ -1044,42 +1003,42 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
+          <t>dashboard, tasks, projects, recruitment, campaigns, documents, video, helpdesk, settings, hr</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09 05:51 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Isha Maji</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>system6thejaingroup@gmail.com</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Systems</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
           <t>dashboard, tasks, projects, recruitment, campaigns, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-09 05:51 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Isha Maji</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>system6thejaingroup@gmail.com</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>Systems</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>dashboard, tasks, projects, recruitment, campaigns, documents, video, helpdesk, settings</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>2026-07-09 05:52 UTC</t>
         </is>
@@ -1118,32 +1077,32 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Shuchandra Das</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>mgr.hr@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, hr, recruitment, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>2026-07-11 09:35 UTC</t>
         </is>
@@ -1182,32 +1141,32 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Sriyans Ruia</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>ai@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Systems</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, settings</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>2026-07-16 04:53 UTC</t>
         </is>
@@ -1246,32 +1205,32 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Khusbu Singh</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>hr@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, hr, recruitment, documents, video, settings</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 09:56 UTC</t>
         </is>
@@ -1310,32 +1269,32 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>PALLABITA GHOSH</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>customercare1@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Post Sales</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, crm, projects, recruitment, campaigns, playbook, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 09:57 UTC</t>
         </is>
@@ -1374,32 +1333,32 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Jit Sen</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>sales.exotica1@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, recruitment, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 09:57 UTC</t>
         </is>
@@ -1438,32 +1397,32 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Ankita Bhandari</t>
         </is>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>legal5@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Legal</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, recruitment, legal, compliance, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 09:57 UTC</t>
         </is>
@@ -1502,32 +1461,32 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Chandan Jha</t>
         </is>
       </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>mgr.accounts@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>Accounts</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, recruitment, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 09:57 UTC</t>
         </is>
@@ -1566,32 +1525,32 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Avishek Das</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>sm.sales4@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>CP Sales</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, crm, projects, recruitment, campaigns, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 09:58 UTC</t>
         </is>
@@ -1630,32 +1589,32 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Anubhav Sarkhel</t>
         </is>
       </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>audit3@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, recruitment, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F38" s="6" t="inlineStr">
+      <c r="F38" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 09:58 UTC</t>
         </is>
@@ -1694,32 +1653,32 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Tanmoy Das</t>
         </is>
       </c>
-      <c r="B40" s="6" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>legal1@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Legal</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, recruitment, legal, compliance, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F40" s="6" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 09:58 UTC</t>
         </is>
@@ -1758,32 +1717,32 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>Samrat Saha</t>
-        </is>
-      </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>sales.dreamvalley1@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, crm, projects, recruitment, campaigns, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F42" s="6" t="inlineStr">
+      <c r="F42" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 09:58 UTC</t>
         </is>
@@ -1822,32 +1781,32 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="inlineStr">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Srestha Sarkar</t>
         </is>
       </c>
-      <c r="B44" s="6" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>legal2@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C44" s="6" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>Legal</t>
         </is>
       </c>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, recruitment, legal, compliance, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F44" s="6" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 09:59 UTC</t>
         </is>
@@ -1886,32 +1845,32 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Md Saif Ali</t>
         </is>
       </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>itsupport@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E46" s="7" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, recruitment, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F46" s="6" t="inlineStr">
+      <c r="F46" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 09:59 UTC</t>
         </is>
@@ -1950,32 +1909,32 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="inlineStr">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>Sukanya Saha</t>
         </is>
       </c>
-      <c r="B48" s="6" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>sales.dwc5@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E48" s="7" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, crm, projects, recruitment, campaigns, playbook, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F48" s="6" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 10:00 UTC</t>
         </is>
@@ -2014,32 +1973,32 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="inlineStr">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>Rabindra Nath Dey</t>
         </is>
       </c>
-      <c r="B50" s="6" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>purchase@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>(not provisioned)</t>
-        </is>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Purchase</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, inventory, procurement, inspection, recruitment, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F50" s="6" t="inlineStr">
+      <c r="F50" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 10:00 UTC</t>
         </is>
@@ -2078,32 +2037,32 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="inlineStr">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>Bachchu Samanta</t>
         </is>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>accounts5@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>Accounts</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="inlineStr">
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, recruitment, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F52" s="6" t="inlineStr">
+      <c r="F52" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 10:01 UTC</t>
         </is>
@@ -2142,32 +2101,32 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>Linisha Saha</t>
         </is>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>system5thejaingroup@gmail.com</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E54" s="7" t="inlineStr">
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, recruitment, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F54" s="6" t="inlineStr">
+      <c r="F54" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 10:02 UTC</t>
         </is>
@@ -2206,32 +2165,32 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="inlineStr">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>Arun kr Pandey</t>
         </is>
       </c>
-      <c r="B56" s="6" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>accounts2@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>Accounts</t>
         </is>
       </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="inlineStr">
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, recruitment, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F56" s="6" t="inlineStr">
+      <c r="F56" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 10:04 UTC</t>
         </is>
@@ -2270,32 +2229,32 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>Rani Das</t>
         </is>
       </c>
-      <c r="B58" s="6" t="inlineStr">
+      <c r="B58" s="4" t="inlineStr">
         <is>
           <t>jaingroupcaller9@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>Pre Sales</t>
         </is>
       </c>
-      <c r="D58" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="inlineStr">
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, recruitment, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F58" s="6" t="inlineStr">
+      <c r="F58" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 10:06 UTC</t>
         </is>
@@ -2334,32 +2293,32 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="inlineStr">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>Abhisek Shaw</t>
         </is>
       </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>mgr.sales@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>CP Sales</t>
         </is>
       </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E60" s="7" t="inlineStr">
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, crm, projects, recruitment, campaigns, documents, video, settings</t>
         </is>
       </c>
-      <c r="F60" s="6" t="inlineStr">
+      <c r="F60" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 10:13 UTC</t>
         </is>
@@ -2398,32 +2357,32 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="inlineStr">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>Rishav Saha</t>
         </is>
       </c>
-      <c r="B62" s="6" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>designer2pc@gmail.com</t>
         </is>
       </c>
-      <c r="C62" s="6" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E62" s="7" t="inlineStr">
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, projects, recruitment, campaigns, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F62" s="6" t="inlineStr">
+      <c r="F62" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 10:26 UTC</t>
         </is>
@@ -2462,32 +2421,32 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="inlineStr">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>Subrata Das</t>
         </is>
       </c>
-      <c r="B64" s="6" t="inlineStr">
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>sales.dreamecocity2@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C64" s="6" t="inlineStr">
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="inlineStr">
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, crm, projects, recruitment, campaigns, documents, video, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F64" s="6" t="inlineStr">
+      <c r="F64" s="4" t="inlineStr">
         <is>
           <t>2026-07-18 12:00 UTC</t>
         </is>
@@ -2526,42 +2485,38 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="inlineStr">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>Biswajit Banerjee</t>
         </is>
       </c>
-      <c r="B66" s="6" t="inlineStr">
+      <c r="B66" s="4" t="inlineStr">
         <is>
           <t>facility@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C66" s="6" t="inlineStr">
+      <c r="C66" s="4" t="inlineStr">
         <is>
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="D66" s="6" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="E66" s="7" t="inlineStr">
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
         <is>
           <t>dashboard, tasks, crm, projects, recruitment, campaigns, documents, helpdesk, settings</t>
         </is>
       </c>
-      <c r="F66" s="6" t="inlineStr">
+      <c r="F66" s="4" t="inlineStr">
         <is>
           <t>2026-07-20 06:19 UTC</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F66"/>
-  <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2593,7 +2548,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-20 10:34 UTC · "Made Tasks" = created at least one task in acc.ptasks (including tasks later deleted, recovered from orphaned acc.notifications rows since acc.ptasks itself has no soft-delete trail) · 125 live tasks across 40 live creators</t>
+          <t>Generated 2026-07-22 06:33 UTC · "Made Tasks" = created at least one task in acc.ptasks (including tasks later deleted, recovered from orphaned acc.notifications rows since acc.ptasks itself has no soft-delete trail) · 165 live+recovered tasks across 46 creators</t>
         </is>
       </c>
     </row>
@@ -2645,59 +2600,59 @@
           <t>Systems, Sales, Marketing, Pre Sales, Post Sales</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Accountability review; Adhoc term replacement feature in JainE for post sales; Claude image generation feedback; Complaint resolution feedback form; Give view access to Shesha of hotel social media; heroku; HR module review in JainE; Inspection review; Integrate meetings into accountability; Internet speed tracker; Knowlarity cli number surrender; Legal module review in JainE; Other LinkedIn posts to be tagged with rishiji; plc flc of ananta; postmark; Recruitment post hr to be tagged; Status matrix of Ananta; Stock aging; Stock aging automation; Task1; Test again; Vendor trend analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Administrator</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>ayushruia1@gmail.com</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Knowlarity cli number surrender; Claude image generation feedback; Complaint resolution feedback form; Recruitment post hr to be tagged; Give view access to Shesha of hotel social media; Other LinkedIn posts to be tagged with rishiji; Status matrix of Ananta; HR module review in JainE; Adhoc term replacement feature in JainE for post sales; Legal module review in JainE; Internet speed tracker; Integrate meetings into accountability; Inspection review; Stock aging; Vendor trend analysis; Stock aging automation; plc flc of ananta; postmark; heroku</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Manash Choudhury</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>digitalmarketing@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>Durbaar Banquets Campaign Video to Complete; Zappier Login Details Required for CAPI Implementation; Booking Form Checking; Claude image generation feedback; Durbaar Banquets - Video Edits; Durbaar - Video Thumbnail to Create; WhatsApp Lead Filtration Feature Similar to Exotica; META CLI to Implement in Linux &amp; Do Research; CRM - Drill Down Report - Google Spend Graph Not Showing; CRM - Ad Wise Facebook Report - Design Issues to Rectify; CRM - Application Error Shown While Checking Lists of Customer Data</t>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>fgrerthtr; H; Hey; Hey yooooo; IDK; Ok; rdtfyuio;; Task 3; Task1; Task2; Task3; Task5</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Riya Dey</t>
+          <t>Manash Choudhury</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>designerthejaingroup@gmail.com</t>
+          <t>digitalmarketing@thejaingroup.com</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -2705,119 +2660,119 @@
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Birthday photo edit and share; DWC EMI and Car Parking creative landscape version resize; Ananta script shot division; DWC car branding; Ananta motion logo audio; Durbaar video edit</t>
+          <t>Booking Form Checking; Claude image generation feedback; CRM - Ad Wise Facebook Report - Design Issues to Rectify; CRM - Application Error Shown While Checking Lists of Customer Data; CRM - Drill Down Report - Google Spend Graph Not Showing; Durbaar - Video Thumbnail to Create; Durbaar Banquets - Video Edits; Durbaar Banquets Campaign Video to Complete; META CLI to Implement in Linux &amp; Do Research; Performance Report Update - Ayush Ji Told Me Over Phone; Test1; WhatsApp Lead Filtration Feature Similar to Exotica; Zappier Login Details Required for CAPI Implementation</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Tanmoy Das</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>legal1@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Legal</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>1st Class Magistrate Affidavit of Sujata Ghosh, Project - A K Mukherjee; Paper Publication Approved by Chairman sir ( Project - Badu III Mutation Purpose); Certified Power Deed No 7440 of 2012 at ADSR Barasat Office (Project - Badu III Mutation Purpose); Dream Ananta Gurukul Quaterly updation - RERA; Badu III - 23 decimal khatian complete within this week; Drafting of 1st magistrate affidavit of Badu iii project for mutation purpose</t>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>1st Class Magistrate Affidavit of Sujata Ghosh, Project - A K Mukherjee; Badu III - 23 decimal khatian complete within this week; Certified Power Deed No 7440 of 2012 at ADSR Barasat Office (Project - Badu III Mutation Purpose); Drafting of 1st magistrate affidavit of Badu iii project for mutation purpose; Dream Ananta Gurukul Quaterly updation - RERA; Mail to RERA Office for quarterly updation, Project - Gurukul. Eco City Block 10, Dwc; Paper Publication Approved by Chairman sir ( Project - Badu III Mutation Purpose); RERA - Dram Eco city Verify and redraft and all documents sent to Director Sir for Approval</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Jiya Das</t>
+          <t>Gokul Saha</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>customercare3@thejaingroup.com</t>
+          <t>ea.md@thejaingroup.com</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Post Sales</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>MAKE QUERY DEED &amp; PAYMENT PLAN FOR REGISTRATION; MAKE QUERY &amp; DEED FOR REGISTRATION; MAKE QUERY &amp; DEED FOR REGISTRATION (MR. &amp; MS. VIDYARATHI); MAKE QUERY &amp; DEED FOR REGISTRATION (MR. &amp; MS. VIDYARATHI); PLEASE APPROVE MY SHORT LEAVE</t>
+          <t>Carpet Tiles set-up HO; GMH H.Inn Insurance preparing cheque; Health Insurance renewal of Mrs.Pramila Ma'am; Park+ implementation work at D.One; Purchasing 5 new Chair; Swimming pool at D.One installing Thermostat</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Sukanya Saha</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>sales.dwc5@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Task1; Task1; Task3; Task 2; Task 6</t>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Riya Dey</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>designerthejaingroup@gmail.com</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Ananta motion logo audio; Ananta script shot division; Birthday photo edit and share; Durbaar video edit; DWC car branding; DWC EMI and Car Parking creative landscape version resize</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>PALLABITA GHOSH</t>
+          <t>Jiya Das</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>customercare1@thejaingroup.com</t>
+          <t>customercare3@thejaingroup.com</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -2825,67 +2780,67 @@
           <t>Post Sales</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Rabi Datta extra work classification; Demand for Ananta to be sent by day end; Mehboob Alam cancellation &amp; refund; Taskforce review for Palazzo &amp; Exotica</t>
+          <t>MAKE QUERY &amp; DEED FOR REGISTRATION; MAKE QUERY &amp; DEED FOR REGISTRATION (MR. &amp; MS. VIDYARATHI); MAKE QUERY DEED &amp; PAYMENT PLAN FOR REGISTRATION; PLEASE APPROVE MY SHORT LEAVE</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Sandip Das</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>marketing@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>PO generation of Stylo; Design creative; Social media calendar creation; CP meeting</t>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Sukanya Saha</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>sales.dwc5@thejaingroup.com</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Task 2; Task 6; Task1; Task3</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Chandan Jha</t>
+          <t>PALLABITA GHOSH</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>mgr.accounts@thejaingroup.com</t>
+          <t>customercare1@thejaingroup.com</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Accounts</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
+          <t>Post Sales</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2895,49 +2850,49 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>test task; test task; Test Task 3; Test Task 4</t>
+          <t>Demand for Ananta to be sent by day end; Mehboob Alam cancellation &amp; refund; Rabi Datta extra work classification; Taskforce review for Palazzo &amp; Exotica</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Santanu Naskar</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>projectmanager1@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="n">
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>JCB approval; Check list; RMC; RMC Approval</t>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Check list; JCB approval; RMC; RMC Approval</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Gyan Prakash Pandey</t>
+          <t>Chandan Jha</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>sm.accounts@thejaingroup.com</t>
+          <t>mgr.accounts@thejaingroup.com</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -2945,7 +2900,7 @@
           <t>Accounts</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2955,117 +2910,117 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>GSTR-3B for June 26; Test; Prepare NBFC Survey -Questionnaire of 3 NBFC companies; Finalize Debit Balance Sheet of Creditors of JGPPL</t>
+          <t>test task; Test Task 3; Test Task 4</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Arun kr Pandey</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>accounts2@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Gyan Prakash Pandey</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>sm.accounts@thejaingroup.com</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Accounts</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>TDS; task3; Bills</t>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Finalize Debit Balance Sheet of Creditors of JGPPL; GSTR-3B for June 26; Prepare NBFC Survey -Questionnaire of 3 NBFC companies; Test</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Santosh Kumar</t>
+          <t>Sandip Das</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>admin.facility@thejaingroup.com</t>
+          <t>marketing@thejaingroup.com</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Administration</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>CP meeting; Design creative; PO generation of Stylo; Social media calendar creation</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Riya Roy</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>customercare2@thejaingroup.com</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Post Sales</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>payment for urgent; bill checking; payment process</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Soumyadeep Guhaneogi</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>audit2@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Legal</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>Mousumi Banerjee Bank Satement dated 10-01-2023, 18-02-2023, and 09-08-2023; The transactions amounting to Rs. 25,00,000.00, Rs. 6,41,904.00, and Rs. 91,030.00, dated 10-01-2023, 18-02-2023, and 09-08-2023, respectively, are not reflected in Mousumi Banerjee's bank statement.; brs</t>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Car parking letter to sign and clear; Make a Details for payment; Want to know the details of DWC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Riya Roy</t>
+          <t>Shuchandra Das</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>customercare2@thejaingroup.com</t>
+          <t>mgr.hr@thejaingroup.com</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Post Sales</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3075,57 +3030,57 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Make a Details for payment; Want to know the details of DWC; Car parking letter to sign and clear</t>
+          <t>Legal executive interview schedule for monday; Process Coordinator interview line up; Sales Manager for Hotel Line up</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Susanta Ghosh</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>gm.commercial@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>Purchase</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="n">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Rima Mandal</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>wecare@thejaingroup.com</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Post Sales</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>Aush Ji ( Stock Ageing Report); Try 2; Carpet Work ..</t>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Arnab Bose Car Parking Number.; Durga Gupta Registry Date; Want To Know Khusi Pandey Left Balance</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Shuchandra Das</t>
+          <t>Bachchu Samanta</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>mgr.hr@thejaingroup.com</t>
+          <t>accounts5@thejaingroup.com</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>HR</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
+          <t>Accounts</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3135,57 +3090,57 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Legal executive interview schedule for monday; Sales Manager for Hotel Line up; Process Coordinator interview line up</t>
+          <t>ERP ENTRY; Test Task</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Avishek Das</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>sm.sales4@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>CP Sales</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="n">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Arun kr Pandey</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>accounts2@thejaingroup.com</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Accounts</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>Send Pre-Launch creative to CP groups; Update on Executive Incentive bill of sanju debnath; Update on pending Incentive and brokerage bill</t>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Bills; task3; TDS</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Rima Mandal</t>
+          <t>Santosh Kumar</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>wecare@thejaingroup.com</t>
+          <t>admin.facility@thejaingroup.com</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Post Sales</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="inlineStr">
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3195,117 +3150,117 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Arnab Bose Car Parking Number.; Durga Gupta Registry Date; Want To Know Khusi Pandey Left Balance</t>
+          <t>bill checking; payment for urgent; payment process</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Bachchu Samanta</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>accounts5@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>Accounts</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>Test Task; Test Task</t>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Soumyadeep Guhaneogi</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>audit2@thejaingroup.com</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>brs; Mousumi Banerjee Bank Satement dated 10-01-2023, 18-02-2023, and 09-08-2023; The transactions amounting to Rs. 25,00,000.00, Rs. 6,41,904.00, and Rs. 91,030.00, dated 10-01-2023, 18-02-2023, and 09-08-2023, respectively, are not reflected in Mousumi Banerjee's bank statement.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Madhurima Chowdhury</t>
+          <t>Susanta Ghosh</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>architect@thejaingroup.com</t>
+          <t>gm.commercial@thejaingroup.com</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Operations</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
+          <t>Purchase</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>AKM working; UPI payment</t>
+          <t>Aush Ji ( Stock Ageing Report); Carpet Work ..; Try 2</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Santanu Goswami</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>dgm.project@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>Operations</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>Roof reapring work; Roof reparing work</t>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Avishek Das</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>sm.sales4@thejaingroup.com</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>CP Sales</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Send Pre-Launch creative to CP groups; Update on Executive Incentive bill of sanju debnath; Update on pending Incentive and brokerage bill</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Gokul Saha</t>
+          <t>Mitrabarun Ghosh</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>ea.md@thejaingroup.com</t>
+          <t>sm.projects1@thejaingroup.com</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Administration</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr">
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3315,57 +3270,57 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Carpet Tiles set-up HO; Purchasing 5 new Chair</t>
+          <t>Checking Bill; Pls  check area of  work roof water proof done  by Lokanth</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Biswajit Banerjee</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>facility@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="n">
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>DWC Bus scheduling; Dwc Bus scheduling</t>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Dwc Bus scheduling; DWC Bus scheduling</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Susmita Sarkar</t>
+          <t>Abhay Mati</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>jaingroupcaller6@thejaingroup.com</t>
+          <t>system1@thejaingroup.com</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Pre Sales</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
+          <t>Systems</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3375,57 +3330,57 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>exotica details add on CRM template; CRM</t>
+          <t>update employee details; update me about the HR module</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>Mitrabarun Ghosh</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>sm.projects1@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>Operations</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="n">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Susmita Sarkar</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>jaingroupcaller6@thejaingroup.com</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Pre Sales</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>Checking Bill; Pls  check area of  work roof water proof done  by Lokanth</t>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>CRM; exotica details add on CRM template</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Linisha Saha</t>
+          <t>Santanu Goswami</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>system5thejaingroup@gmail.com</t>
+          <t>dgm.project@thejaingroup.com</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3435,169 +3390,169 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Bullseye Video Edit; Skizzel update</t>
+          <t>Roof reapring work; Roof reparing work</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>Uzma Ahmed</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>career@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>HR</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>Sales Manager Interview</t>
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Vicky Mallick</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>system3.thejaingroup@gmail.com</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Systems</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Farvision mongo db auto shutting down; farvision test</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Rishav Saha</t>
+          <t>Prerna Gupta</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>designer2pc@gmail.com</t>
+          <t>businessanalyst@thejaingroup.com</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
+          <t>Systems</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Research for aesthetics</t>
+          <t>Stock aging automation; Task2</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>Amirul SK</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>graphicsdesinger3.thejaingroup@gmail.com</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="D34" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>Claude image generation feedback</t>
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Madhurima Chowdhury</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>architect@thejaingroup.com</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>AKM working; UPI payment</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Khusbu Singh</t>
+          <t>Linisha Saha</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>hr@thejaingroup.com</t>
+          <t>system5thejaingroup@gmail.com</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>HR</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Legal Interview -Follow up</t>
+          <t>Bullseye Video Edit; Skizzel update</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>Srestha Sarkar</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>legal2@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Ankita Bhandari</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>legal5@thejaingroup.com</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Legal</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="7" t="inlineStr">
-        <is>
-          <t>Drafting of reply</t>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>A query deed for registration needs to be prepared for a Dream One customer by Monday.; DWC SAIKAT BERA QUERY &amp; DEED READY</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Ankita Bhandari</t>
+          <t>Srestha Sarkar</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>legal5@thejaingroup.com</t>
+          <t>legal2@thejaingroup.com</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -3605,7 +3560,7 @@
           <t>Legal</t>
         </is>
       </c>
-      <c r="D37" s="8" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3615,57 +3570,57 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>A query deed for registration needs to be prepared for a Dream One customer by Monday.</t>
+          <t>Drafting of reply</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>Dipanwita Chatterjee</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>mgr.presales@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>Pre Sales</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="n">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Mukesh kr. Laheri</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>mukesh@thejaingroup.com</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F38" s="7" t="inlineStr">
-        <is>
-          <t>CRM</t>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>mongo update</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Abhisek Shaw</t>
+          <t>Akashnil Basu</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>mgr.sales@thejaingroup.com</t>
+          <t>socialmedia@thejaingroup.com</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>CP Sales</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3675,57 +3630,57 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>need agreement for</t>
+          <t>ngvgfhmhgcghf</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>Mukesh kr. Laheri</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>mukesh@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="n">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Amirul SK</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>graphicsdesinger3.thejaingroup@gmail.com</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>mongo update</t>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Claude image generation feedback</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Sanhita Mukherjee</t>
+          <t>Isha Maji</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>pr1@thejaingroup.com</t>
+          <t>system6thejaingroup@gmail.com</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
+          <t>Systems</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3735,49 +3690,49 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>skizzle update</t>
+          <t>test task</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>Dibas Shyamal</t>
-        </is>
-      </c>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>system2.thejaingroup@gmail.com</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>Systems</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="n">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Rishav Saha</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>designer2pc@gmail.com</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F42" s="7" t="inlineStr">
-        <is>
-          <t>Please check fervision AWS backup</t>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Research for aesthetics</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Vicky Mallick</t>
+          <t>Sriyans Ruia</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>system3.thejaingroup@gmail.com</t>
+          <t>ai@thejaingroup.com</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -3785,7 +3740,7 @@
           <t>Systems</t>
         </is>
       </c>
-      <c r="D43" s="8" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3795,177 +3750,177 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>farvision test</t>
+          <t>Task1</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>Isha Maji</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>system6thejaingroup@gmail.com</t>
-        </is>
-      </c>
-      <c r="C44" s="6" t="inlineStr">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dibas Shyamal</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>system2.thejaingroup@gmail.com</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>Systems</t>
         </is>
       </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="n">
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F44" s="7" t="inlineStr">
-        <is>
-          <t>test task</t>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Please check fervision AWS backup</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Khusbu Singh</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>ayushruia1@gmail.com</t>
+          <t>hr@thejaingroup.com</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Administration</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Hey yooooo; fgrerthtr; rdtfyuio;; Task1; Task2; Hey; Task3; Ok; Hey; IDK; Task1; Task2; Task 3; Task5; Ok; Task1; Task2; Task3</t>
+          <t>Legal Interview -Follow up</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>Akashnil Basu</t>
-        </is>
-      </c>
-      <c r="B46" s="6" t="inlineStr">
-        <is>
-          <t>socialmedia@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C46" s="6" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>Task3; ngvgfhmhgcghf</t>
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Uzma Ahmed</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>career@thejaingroup.com</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Sales Manager Interview</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Prerna Gupta</t>
+          <t>Abhisek Shaw</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>businessanalyst@thejaingroup.com</t>
+          <t>mgr.sales@thejaingroup.com</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Systems</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
+          <t>CP Sales</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="E47" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Task2; Stock aging automation</t>
+          <t>need agreement for</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>Abhay Mati</t>
-        </is>
-      </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>system1@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C48" s="6" t="inlineStr">
-        <is>
-          <t>Systems</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E48" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F48" s="7" t="inlineStr">
-        <is>
-          <t>update me about the HR module; update employee details</t>
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Dipanwita Chatterjee</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>mgr.presales@thejaingroup.com</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Pre Sales</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>CRM</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Sriyans Ruia</t>
+          <t>Miraj Ahmed</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>ai@thejaingroup.com</t>
+          <t>sales.dwc2@thejaingroup.com</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Systems</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3975,37 +3930,37 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Task1</t>
+          <t>reement</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>Miraj Ahmed</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>sales.dwc2@thejaingroup.com</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="n">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Sanhita Mukherjee</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>pr1@thejaingroup.com</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F50" s="7" t="inlineStr">
-        <is>
-          <t>agreement</t>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>skizzle update</t>
         </is>
       </c>
     </row>
@@ -4025,7 +3980,7 @@
           <t>Finance</t>
         </is>
       </c>
-      <c r="D51" s="9" t="inlineStr">
+      <c r="D51" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4033,33 +3988,31 @@
       <c r="E51" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="inlineStr">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>Arhum Alam</t>
         </is>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>engineer6jaingroup@gmail.com</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D52" s="9" t="inlineStr">
+      <c r="D52" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E52" s="6" t="n">
+      <c r="E52" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F52" s="7" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -4077,7 +4030,7 @@
           <t>Sales</t>
         </is>
       </c>
-      <c r="D53" s="9" t="inlineStr">
+      <c r="D53" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4085,33 +4038,31 @@
       <c r="E53" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>Dhrubajyoti Adhikary</t>
         </is>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>sm.sales2@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D54" s="9" t="inlineStr">
+      <c r="D54" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E54" s="6" t="n">
+      <c r="E54" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F54" s="7" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -4129,7 +4080,7 @@
           <t>Accounts</t>
         </is>
       </c>
-      <c r="D55" s="9" t="inlineStr">
+      <c r="D55" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4137,33 +4088,31 @@
       <c r="E55" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="inlineStr">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>Jit Sen</t>
         </is>
       </c>
-      <c r="B56" s="6" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>sales.exotica1@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D56" s="9" t="inlineStr">
+      <c r="D56" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E56" s="6" t="n">
+      <c r="E56" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F56" s="7" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -4181,7 +4130,7 @@
           <t>IT</t>
         </is>
       </c>
-      <c r="D57" s="9" t="inlineStr">
+      <c r="D57" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4189,33 +4138,31 @@
       <c r="E57" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>Rabindra Nath Dey</t>
         </is>
       </c>
-      <c r="B58" s="6" t="inlineStr">
+      <c r="B58" s="4" t="inlineStr">
         <is>
           <t>purchase@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D58" s="9" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Purchase</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E58" s="6" t="n">
+      <c r="E58" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F58" s="7" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -4233,7 +4180,7 @@
           <t>Pre Sales</t>
         </is>
       </c>
-      <c r="D59" s="9" t="inlineStr">
+      <c r="D59" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4241,33 +4188,31 @@
       <c r="E59" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="inlineStr">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>Rishi Jain</t>
         </is>
       </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>rishi@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>Management</t>
         </is>
       </c>
-      <c r="D60" s="9" t="inlineStr">
+      <c r="D60" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E60" s="6" t="n">
+      <c r="E60" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F60" s="7" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -4285,7 +4230,7 @@
           <t>Sales</t>
         </is>
       </c>
-      <c r="D61" s="9" t="inlineStr">
+      <c r="D61" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4293,33 +4238,31 @@
       <c r="E61" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F61" s="5" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t>Samrat Saha</t>
-        </is>
-      </c>
-      <c r="B62" s="6" t="inlineStr">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>sales.dreamvalley1</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>sales.dreamvalley1@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C62" s="6" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D62" s="9" t="inlineStr">
+      <c r="D62" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E62" s="6" t="n">
+      <c r="E62" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F62" s="7" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -4337,7 +4280,7 @@
           <t>Finance</t>
         </is>
       </c>
-      <c r="D63" s="9" t="inlineStr">
+      <c r="D63" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4345,33 +4288,31 @@
       <c r="E63" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="inlineStr">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>Subrata Das</t>
         </is>
       </c>
-      <c r="B64" s="6" t="inlineStr">
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>sales.dreamecocity2@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C64" s="6" t="inlineStr">
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D64" s="9" t="inlineStr">
+      <c r="D64" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E64" s="6" t="n">
+      <c r="E64" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F64" s="7" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -4389,7 +4330,7 @@
           <t>HR</t>
         </is>
       </c>
-      <c r="D65" s="9" t="inlineStr">
+      <c r="D65" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4397,39 +4338,33 @@
       <c r="E65" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="inlineStr">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>v c</t>
         </is>
       </c>
-      <c r="B66" s="6" t="inlineStr">
+      <c r="B66" s="4" t="inlineStr">
         <is>
           <t>vc@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C66" s="6" t="inlineStr">
+      <c r="C66" s="4" t="inlineStr">
         <is>
           <t>Management</t>
         </is>
       </c>
-      <c r="D66" s="9" t="inlineStr">
+      <c r="D66" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E66" s="6" t="n">
+      <c r="E66" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F66" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F66"/>
-  <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4460,50 +4395,50 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-20 10:34 UTC · based on doc.documents (department = Legal) — the only activity trail available; JAIN-E does not log page views, so document uploads are the only detectable signal of someone actually using the Legal page.</t>
+          <t>Generated 2026-07-22 06:33 UTC · based on doc.documents (department = Legal) — the only activity trail available; JAIN-E does not log page views, so document uploads are the only detectable signal of someone actually using the Legal page.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>1. Has a new document been uploaded to Legal recently?</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Last document uploaded: 2026-07-07 05:36 UTC (13 days before this report). Nothing has been uploaded since. Total documents in the Legal vault: 786, all uploaded between 2026-07-04 and 2026-07-07.</t>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Last document uploaded: 2026-07-07 05:36 UTC (15 days before this report). Nothing has been uploaded since. Total documents in the Legal vault: 786, all uploaded between 2026-07-04 and 2026-07-07.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>2. Has any user other than the Administrator used the Legal page?</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="75" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Every one of the 786 Legal documents was uploaded under a single account — digitalmarketing@thejaingroup.com (Manash Choudhury) — not the Administrator account (ayushruia1@gmail.com). All 786 were uploaded in a 3-day window (2026-07-04 to 2026-07-07), before this account even had "legal" module access on its profile — this points to a one-time bulk import/migration, not day-to-day use of the Legal page. No document has ever been uploaded by the Administrator, and none of the 4 people in the Legal department have uploaded anything (see table below).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Who has ever uploaded to Legal</t>
         </is>
@@ -4537,32 +4472,32 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>digitalmarketing@thejaingroup.com</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Manash Choudhury</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="10" t="n">
         <v>786</v>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>2026-07-04 11:30 UTC</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>2026-07-07 05:36 UTC</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Legal-department members provisioned in JAIN-E</t>
         </is>
@@ -4596,113 +4531,106 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Ankita Bhandari</t>
         </is>
       </c>
-      <c r="B16" s="14" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>legal5@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="n">
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="15" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Soumyadeep Guhaneogi</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>audit2@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D17" s="14" t="n">
+      <c r="D17" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Srestha Sarkar</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>legal2@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="n">
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="15" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Tanmoy Das</t>
         </is>
       </c>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>legal1@thejaingroup.com</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="n">
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="15" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="B5:E5"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>